<commit_message>
Update to data dictionary, ignore if you want
</commit_message>
<xml_diff>
--- a/Documentation/Photos/Data Dictionary.xlsx
+++ b/Documentation/Photos/Data Dictionary.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30215"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBD1FA50-2EAA-4115-8574-D8684C39E13C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F51F6D6-833E-4B24-8A3D-894C313219B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Variables" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="328">
   <si>
     <t>Variable Name</t>
   </si>
@@ -77,7 +77,7 @@
     <t>private</t>
   </si>
   <si>
-    <t>Class</t>
+    <t>Class (GameManager)</t>
   </si>
   <si>
     <t>variables, methods</t>
@@ -413,7 +413,7 @@
     <t>Vector2Int, string</t>
   </si>
   <si>
-    <t>{V2Int : string, V2Int : string, ..., V2Int : string, V2Int : string}</t>
+    <t>{V2Int : S, V2Int : S, ..., V2Int : S, V2Int : S}</t>
   </si>
   <si>
     <t>GenerateMap</t>
@@ -422,6 +422,150 @@
     <t>mapSpawnEdge^, mapBossSpawn^</t>
   </si>
   <si>
+    <t>coinController</t>
+  </si>
+  <si>
+    <t>The AssembledCoinController script</t>
+  </si>
+  <si>
+    <t>Class (AssembledCoinController)</t>
+  </si>
+  <si>
+    <t>PlayerController</t>
+  </si>
+  <si>
+    <t>Awake, AddToInventory</t>
+  </si>
+  <si>
+    <t>other^</t>
+  </si>
+  <si>
+    <t>Awake, Update</t>
+  </si>
+  <si>
+    <t>hit^</t>
+  </si>
+  <si>
+    <t>moveAction</t>
+  </si>
+  <si>
+    <t>The move action system of the Player</t>
+  </si>
+  <si>
+    <t>Class (InputAction)</t>
+  </si>
+  <si>
+    <t>Start, Update</t>
+  </si>
+  <si>
+    <t>move</t>
+  </si>
+  <si>
+    <t>rigidbody2d</t>
+  </si>
+  <si>
+    <t>The Rigidbody2D component of the Player</t>
+  </si>
+  <si>
+    <t>Class (Rigidbody2D)</t>
+  </si>
+  <si>
+    <t>Awake, Update, FixedUpdate</t>
+  </si>
+  <si>
+    <t>hit^, moveDirection, move, speed, position^</t>
+  </si>
+  <si>
+    <t>The movement of the player</t>
+  </si>
+  <si>
+    <t>Vector2</t>
+  </si>
+  <si>
+    <t>Update, FixedUpdate</t>
+  </si>
+  <si>
+    <t>moveAction, moveDirection, animator, position, rigidbody2d, speed</t>
+  </si>
+  <si>
+    <t>InteractAction</t>
+  </si>
+  <si>
+    <t>The interact action of system of the Player</t>
+  </si>
+  <si>
+    <t>talkInteractions</t>
+  </si>
+  <si>
+    <t>List of interactions to talk to</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>[S, S, ..., S, S]</t>
+  </si>
+  <si>
+    <t>Update</t>
+  </si>
+  <si>
+    <t>changeIterations</t>
+  </si>
+  <si>
+    <t>List of interactions to change something</t>
+  </si>
+  <si>
+    <t>inspectIterations</t>
+  </si>
+  <si>
+    <t>List of iteractions to inspect something</t>
+  </si>
+  <si>
+    <t>timeInvincible</t>
+  </si>
+  <si>
+    <t>The amount of time that the Player is invincible</t>
+  </si>
+  <si>
+    <t>ChangeHealth</t>
+  </si>
+  <si>
+    <t>amount^, damageCooldown</t>
+  </si>
+  <si>
+    <t>isInvincible</t>
+  </si>
+  <si>
+    <t>Whether the Player is invincible</t>
+  </si>
+  <si>
+    <t>Update, ChangeHealth</t>
+  </si>
+  <si>
+    <t>damageCooldown, amount^, timeInvincible</t>
+  </si>
+  <si>
+    <t>damageCooldown</t>
+  </si>
+  <si>
+    <t>The time for the Player's i-frames</t>
+  </si>
+  <si>
+    <t>isInvincible, timeInvincible</t>
+  </si>
+  <si>
+    <t>inventory</t>
+  </si>
+  <si>
+    <t>The player's inventory</t>
+  </si>
+  <si>
+    <t>Update, AddToInventory</t>
+  </si>
+  <si>
+    <t>hit^, minotaurDirection^, other^</t>
+  </si>
+  <si>
     <t>Declaration Method</t>
   </si>
   <si>
@@ -806,6 +950,63 @@
     <t>roomCoord, translateFactor</t>
   </si>
   <si>
+    <t>hit</t>
+  </si>
+  <si>
+    <t>The raycast sent by the Player</t>
+  </si>
+  <si>
+    <t>Class (RaycastHit2D)</t>
+  </si>
+  <si>
+    <t>rigidbody2d^, moveDirection^, talkInteractions^, changeInteractions^, minotaurScript, minotaurAnimator, minotaurDirection, inventory^, inspectInteractions, interactAction</t>
+  </si>
+  <si>
+    <t>minotaurScript</t>
+  </si>
+  <si>
+    <t>The minotaur GameObject's Minotaur script</t>
+  </si>
+  <si>
+    <t>Class (Minotaur)</t>
+  </si>
+  <si>
+    <t>hit, minotaurDirection, inventory^</t>
+  </si>
+  <si>
+    <t>minotaurAnimator</t>
+  </si>
+  <si>
+    <t>The minotaur GameObject's Animator</t>
+  </si>
+  <si>
+    <t>Class (Animator)</t>
+  </si>
+  <si>
+    <t>hit, minotaurDirection</t>
+  </si>
+  <si>
+    <t>minotaurDirection</t>
+  </si>
+  <si>
+    <t>The minotaur's current direction</t>
+  </si>
+  <si>
+    <t>(F, F)</t>
+  </si>
+  <si>
+    <t>minotaurScript, hit, inventory^</t>
+  </si>
+  <si>
+    <t>FixedUpdate</t>
+  </si>
+  <si>
+    <t>The position for the rigidbody2d to attempt to move to</t>
+  </si>
+  <si>
+    <t>rigidbody2d^, move^, speed^</t>
+  </si>
+  <si>
     <t>Abbreviation</t>
   </si>
   <si>
@@ -819,9 +1020,6 @@
   </si>
   <si>
     <t>S</t>
-  </si>
-  <si>
-    <t>string</t>
   </si>
   <si>
     <t>integer</t>
@@ -1324,8 +1522,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78156BB9-5F0A-45FB-9F1E-52D67683ECE9}" name="Table1" displayName="Table1" ref="A1:J23" totalsRowShown="0">
-  <autoFilter ref="A1:J23" xr:uid="{78156BB9-5F0A-45FB-9F1E-52D67683ECE9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78156BB9-5F0A-45FB-9F1E-52D67683ECE9}" name="Table1" displayName="Table1" ref="A1:J36" totalsRowShown="0">
+  <autoFilter ref="A1:J36" xr:uid="{78156BB9-5F0A-45FB-9F1E-52D67683ECE9}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{1293AFC3-05F4-42CB-A632-0C60EBC9EC44}" name="Variable Name" dataDxfId="18"/>
     <tableColumn id="2" xr3:uid="{A3A3895F-7036-4493-AC76-9390796632C7}" name="Description" dataDxfId="17"/>
@@ -1343,8 +1541,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6F95C47A-AA39-4102-A385-A49746737BEC}" name="Table14" displayName="Table14" ref="A1:I49" totalsRowShown="0">
-  <autoFilter ref="A1:I49" xr:uid="{78156BB9-5F0A-45FB-9F1E-52D67683ECE9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6F95C47A-AA39-4102-A385-A49746737BEC}" name="Table14" displayName="Table14" ref="A1:I54" totalsRowShown="0">
+  <autoFilter ref="A1:I54" xr:uid="{78156BB9-5F0A-45FB-9F1E-52D67683ECE9}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{EEB83C6B-1A5D-46C4-B6A0-248D06D526B7}" name="Variable Name" dataDxfId="8"/>
     <tableColumn id="9" xr3:uid="{45E49A2D-0E71-4F1F-B516-09A663D032D9}" name="Declaration Method" dataDxfId="7"/>
@@ -1668,7 +1866,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
@@ -2430,6 +2628,402 @@
         <v>121</v>
       </c>
     </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10">
+      <c r="A33" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="A34" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
+      <c r="A35" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
+      <c r="A36" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2440,13 +3034,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ECA0923-3D01-4B12-A34B-A7BE61697392}">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.42578125" customWidth="1"/>
     <col min="3" max="3" width="54" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="35.7109375" bestFit="1" customWidth="1"/>
@@ -2459,7 +3053,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>122</v>
+        <v>170</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -2480,18 +3074,18 @@
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>123</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="4" t="s">
-        <v>124</v>
+        <v>172</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>125</v>
+        <v>173</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>126</v>
+        <v>174</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>97</v>
@@ -2500,7 +3094,7 @@
         <v>62</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>89</v>
@@ -2515,13 +3109,13 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="7" t="s">
-        <v>128</v>
+        <v>176</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>120</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>129</v>
+        <v>177</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>21</v>
@@ -2539,7 +3133,7 @@
         <v>15</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>130</v>
+        <v>178</v>
       </c>
       <c r="K3" t="s">
         <v>27</v>
@@ -2547,13 +3141,13 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="7" t="s">
-        <v>131</v>
+        <v>179</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>120</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>132</v>
+        <v>180</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>21</v>
@@ -2571,7 +3165,7 @@
         <v>15</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>133</v>
+        <v>181</v>
       </c>
       <c r="K4" t="s">
         <v>31</v>
@@ -2579,13 +3173,13 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="7" t="s">
-        <v>134</v>
+        <v>182</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>52</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>135</v>
+        <v>183</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>97</v>
@@ -2603,7 +3197,7 @@
         <v>15</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>136</v>
+        <v>184</v>
       </c>
       <c r="K5" t="s">
         <v>40</v>
@@ -2611,13 +3205,13 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="7" t="s">
-        <v>137</v>
+        <v>185</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>52</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>138</v>
+        <v>186</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>21</v>
@@ -2635,21 +3229,21 @@
         <v>15</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>139</v>
+        <v>187</v>
       </c>
       <c r="K6" t="s">
-        <v>140</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="7" t="s">
-        <v>141</v>
+        <v>189</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>52</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>142</v>
+        <v>190</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>87</v>
@@ -2667,18 +3261,18 @@
         <v>15</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>143</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="7" t="s">
-        <v>144</v>
+        <v>192</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>145</v>
+        <v>193</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>97</v>
@@ -2687,7 +3281,7 @@
         <v>62</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>89</v>
@@ -2696,36 +3290,36 @@
         <v>15</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>146</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="7" t="s">
-        <v>147</v>
+        <v>195</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>148</v>
+        <v>196</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>149</v>
+        <v>197</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>150</v>
+        <v>198</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>15</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>152</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2733,10 +3327,10 @@
         <v>100</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>148</v>
+        <v>196</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>153</v>
+        <v>201</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>97</v>
@@ -2745,7 +3339,7 @@
         <v>62</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>89</v>
@@ -2754,18 +3348,18 @@
         <v>15</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>147</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="7" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>155</v>
+        <v>203</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>87</v>
@@ -2774,7 +3368,7 @@
         <v>62</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>89</v>
@@ -2783,18 +3377,18 @@
         <v>15</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>156</v>
+        <v>204</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="7" t="s">
-        <v>157</v>
+        <v>205</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>158</v>
+        <v>206</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>87</v>
@@ -2803,7 +3397,7 @@
         <v>62</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>159</v>
+        <v>207</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>89</v>
@@ -2812,18 +3406,18 @@
         <v>15</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>160</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="7" t="s">
-        <v>144</v>
+        <v>192</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>145</v>
+        <v>193</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>97</v>
@@ -2832,7 +3426,7 @@
         <v>62</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>89</v>
@@ -2841,18 +3435,18 @@
         <v>15</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>161</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="7" t="s">
-        <v>162</v>
+        <v>210</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>163</v>
+        <v>211</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>21</v>
@@ -2870,7 +3464,7 @@
         <v>15</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>164</v>
+        <v>212</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2881,7 +3475,7 @@
         <v>57</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>165</v>
+        <v>213</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>21</v>
@@ -2890,7 +3484,7 @@
         <v>22</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>166</v>
+        <v>214</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>24</v>
@@ -2899,18 +3493,18 @@
         <v>15</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>162</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="7" t="s">
-        <v>167</v>
+        <v>215</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>168</v>
+        <v>216</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>21</v>
@@ -2928,18 +3522,18 @@
         <v>15</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>169</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="7" t="s">
-        <v>170</v>
+        <v>218</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>171</v>
+        <v>219</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>21</v>
@@ -2957,18 +3551,18 @@
         <v>15</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>172</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="7" t="s">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>174</v>
+        <v>222</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>21</v>
@@ -2977,7 +3571,7 @@
         <v>62</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>175</v>
+        <v>223</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>64</v>
@@ -2986,18 +3580,18 @@
         <v>15</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="7" t="s">
-        <v>177</v>
+        <v>225</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>178</v>
+        <v>226</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>21</v>
@@ -3015,18 +3609,18 @@
         <v>15</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>179</v>
+        <v>227</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="7" t="s">
-        <v>161</v>
+        <v>209</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>180</v>
+        <v>228</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>97</v>
@@ -3035,7 +3629,7 @@
         <v>62</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>89</v>
@@ -3044,18 +3638,18 @@
         <v>15</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>181</v>
+        <v>229</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="7" t="s">
-        <v>182</v>
+        <v>230</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>183</v>
+        <v>231</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>21</v>
@@ -3073,47 +3667,47 @@
         <v>15</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>184</v>
+        <v>232</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="7" t="s">
-        <v>185</v>
+        <v>233</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>186</v>
+        <v>234</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>150</v>
+        <v>198</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>159</v>
+        <v>207</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>15</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>187</v>
+        <v>235</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="7" t="s">
-        <v>144</v>
+        <v>192</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>145</v>
+        <v>193</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>97</v>
@@ -3122,7 +3716,7 @@
         <v>62</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>89</v>
@@ -3131,18 +3725,18 @@
         <v>15</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>188</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="7" t="s">
-        <v>189</v>
+        <v>237</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>190</v>
+        <v>238</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>87</v>
@@ -3151,7 +3745,7 @@
         <v>62</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>159</v>
+        <v>207</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>89</v>
@@ -3160,18 +3754,18 @@
         <v>15</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>191</v>
+        <v>239</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="7" t="s">
-        <v>192</v>
+        <v>240</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>193</v>
+        <v>241</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>21</v>
@@ -3189,7 +3783,7 @@
         <v>15</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>194</v>
+        <v>242</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -3200,7 +3794,7 @@
         <v>16</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>165</v>
+        <v>213</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>21</v>
@@ -3218,18 +3812,18 @@
         <v>15</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>195</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="7" t="s">
-        <v>196</v>
+        <v>244</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>197</v>
+        <v>245</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>87</v>
@@ -3238,7 +3832,7 @@
         <v>62</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>89</v>
@@ -3247,18 +3841,18 @@
         <v>15</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>198</v>
+        <v>246</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="7" t="s">
-        <v>167</v>
+        <v>215</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>199</v>
+        <v>247</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>21</v>
@@ -3276,18 +3870,18 @@
         <v>15</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>200</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="7" t="s">
-        <v>170</v>
+        <v>218</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>171</v>
+        <v>219</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>21</v>
@@ -3305,18 +3899,18 @@
         <v>15</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>201</v>
+        <v>249</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="7" t="s">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>174</v>
+        <v>222</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>21</v>
@@ -3334,18 +3928,18 @@
         <v>15</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>202</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="7" t="s">
-        <v>203</v>
+        <v>251</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>204</v>
+        <v>252</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>21</v>
@@ -3363,18 +3957,18 @@
         <v>15</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>205</v>
+        <v>253</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="7" t="s">
-        <v>206</v>
+        <v>254</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>204</v>
+        <v>252</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>21</v>
@@ -3392,18 +3986,18 @@
         <v>15</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>207</v>
+        <v>255</v>
       </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="7" t="s">
-        <v>177</v>
+        <v>225</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>178</v>
+        <v>226</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>21</v>
@@ -3421,18 +4015,18 @@
         <v>15</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>208</v>
+        <v>256</v>
       </c>
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="7" t="s">
-        <v>209</v>
+        <v>257</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>210</v>
+        <v>258</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>87</v>
@@ -3441,7 +4035,7 @@
         <v>62</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>89</v>
@@ -3450,18 +4044,18 @@
         <v>15</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>211</v>
+        <v>259</v>
       </c>
     </row>
     <row r="35" spans="1:9">
       <c r="A35" s="7" t="s">
-        <v>161</v>
+        <v>209</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>180</v>
+        <v>228</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>97</v>
@@ -3470,7 +4064,7 @@
         <v>62</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>89</v>
@@ -3479,18 +4073,18 @@
         <v>15</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>212</v>
+        <v>260</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" s="7" t="s">
-        <v>182</v>
+        <v>230</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>183</v>
+        <v>231</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>21</v>
@@ -3508,18 +4102,18 @@
         <v>15</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>184</v>
+        <v>232</v>
       </c>
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="7" t="s">
-        <v>213</v>
+        <v>261</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>214</v>
+        <v>262</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>21</v>
@@ -3537,7 +4131,7 @@
         <v>15</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>215</v>
+        <v>263</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -3545,10 +4139,10 @@
         <v>95</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>216</v>
+        <v>264</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>217</v>
+        <v>265</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>97</v>
@@ -3566,18 +4160,18 @@
         <v>15</v>
       </c>
       <c r="I38" s="8" t="s">
-        <v>218</v>
+        <v>266</v>
       </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="7" t="s">
-        <v>219</v>
+        <v>267</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>216</v>
+        <v>264</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>220</v>
+        <v>268</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>21</v>
@@ -3595,36 +4189,36 @@
         <v>15</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>221</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="7" t="s">
-        <v>222</v>
+        <v>270</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>216</v>
+        <v>264</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>223</v>
+        <v>271</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>224</v>
+        <v>272</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>62</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>225</v>
+        <v>273</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>226</v>
+        <v>274</v>
       </c>
       <c r="H40" s="5" t="s">
         <v>15</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>227</v>
+        <v>275</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -3632,10 +4226,10 @@
         <v>95</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>228</v>
+        <v>276</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>229</v>
+        <v>277</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>97</v>
@@ -3644,7 +4238,7 @@
         <v>62</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>64</v>
@@ -3653,7 +4247,7 @@
         <v>15</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>230</v>
+        <v>278</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -3661,10 +4255,10 @@
         <v>95</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>231</v>
+        <v>279</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>229</v>
+        <v>277</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>97</v>
@@ -3673,7 +4267,7 @@
         <v>62</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>64</v>
@@ -3682,18 +4276,18 @@
         <v>15</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>232</v>
+        <v>280</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" s="4" t="s">
-        <v>233</v>
+        <v>281</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>231</v>
+        <v>279</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>234</v>
+        <v>282</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>21</v>
@@ -3711,18 +4305,18 @@
         <v>15</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>235</v>
+        <v>283</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="4" t="s">
-        <v>236</v>
+        <v>284</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>231</v>
+        <v>279</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>237</v>
+        <v>285</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>97</v>
@@ -3731,7 +4325,7 @@
         <v>62</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>127</v>
+        <v>175</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>64</v>
@@ -3740,7 +4334,7 @@
         <v>15</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>238</v>
+        <v>286</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -3748,10 +4342,10 @@
         <v>91</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>239</v>
+        <v>287</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>240</v>
+        <v>288</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>87</v>
@@ -3769,18 +4363,18 @@
         <v>15</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>241</v>
+        <v>289</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" s="7" t="s">
-        <v>242</v>
+        <v>290</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>239</v>
+        <v>287</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>243</v>
+        <v>291</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>21</v>
@@ -3798,18 +4392,18 @@
         <v>15</v>
       </c>
       <c r="I46" s="8" t="s">
-        <v>244</v>
+        <v>292</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" s="7" t="s">
-        <v>241</v>
+        <v>289</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>239</v>
+        <v>287</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>245</v>
+        <v>293</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>21</v>
@@ -3827,18 +4421,18 @@
         <v>15</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>246</v>
+        <v>294</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" s="7" t="s">
-        <v>242</v>
+        <v>290</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>247</v>
+        <v>295</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>243</v>
+        <v>291</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>21</v>
@@ -3856,18 +4450,18 @@
         <v>15</v>
       </c>
       <c r="I48" s="8" t="s">
-        <v>248</v>
+        <v>296</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" s="7" t="s">
-        <v>241</v>
+        <v>289</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>247</v>
+        <v>295</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>245</v>
+        <v>293</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>21</v>
@@ -3885,7 +4479,140 @@
         <v>15</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>249</v>
+        <v>297</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I50" s="6" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -3907,26 +4634,26 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>250</v>
+        <v>317</v>
       </c>
       <c r="B1" t="s">
-        <v>251</v>
+        <v>318</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>252</v>
+        <v>319</v>
       </c>
       <c r="B2" t="s">
-        <v>253</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>254</v>
+        <v>321</v>
       </c>
       <c r="B3" t="s">
-        <v>255</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -3934,7 +4661,7 @@
         <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>256</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -3947,15 +4674,15 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>257</v>
+        <v>323</v>
       </c>
       <c r="B6" t="s">
-        <v>258</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>259</v>
+        <v>325</v>
       </c>
       <c r="B7" t="s">
         <v>21</v>
@@ -3966,12 +4693,12 @@
         <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>260</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>261</v>
+        <v>327</v>
       </c>
       <c r="B9" t="s">
         <v>62</v>

</xml_diff>